<commit_message>
Fix the download response
</commit_message>
<xml_diff>
--- a/public/monthName_year.xlsx
+++ b/public/monthName_year.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="40">
   <si>
     <t>STATUS OF LEAVE CREDITS</t>
   </si>
@@ -102,15 +102,64 @@
     <t>complete submission with attachments</t>
   </si>
   <si>
-    <t>Test User</t>
-  </si>
-  <si>
-    <t>Feb 3, 27 mins T
-Feb 8, 26 mins T
-Feb 11, 11 mins T</t>
-  </si>
-  <si>
-    <t>Feb 9 - VL</t>
+    <t>Ray Francis Alingasa</t>
+  </si>
+  <si>
+    <t>Jenn Eric Borday</t>
+  </si>
+  <si>
+    <t>Ronald Anthony Briol</t>
+  </si>
+  <si>
+    <t>Marc Gil Calang</t>
+  </si>
+  <si>
+    <t>Rosalie Carpizo</t>
+  </si>
+  <si>
+    <t>Lorene Catedral</t>
+  </si>
+  <si>
+    <t>Carlito Jr. Clarete</t>
+  </si>
+  <si>
+    <t>Kim Durango</t>
+  </si>
+  <si>
+    <t>Jayvee Gustilo</t>
+  </si>
+  <si>
+    <t>Aizy Lyn Joloyohoy</t>
+  </si>
+  <si>
+    <t>Ryan Joloyohoy</t>
+  </si>
+  <si>
+    <t>Diana Lim</t>
+  </si>
+  <si>
+    <t>Dave Madayag</t>
+  </si>
+  <si>
+    <t>Georiss Mae Maniago</t>
+  </si>
+  <si>
+    <t>Amado Posas</t>
+  </si>
+  <si>
+    <t>April Rose Anne Sanchez-Elmedulan</t>
+  </si>
+  <si>
+    <t>Marie Lynn Tadle</t>
+  </si>
+  <si>
+    <t>John Lenn Uayan</t>
+  </si>
+  <si>
+    <t>Grace Villanueva</t>
+  </si>
+  <si>
+    <t>Angelic Mae Yu</t>
   </si>
 </sst>
 </file>
@@ -898,31 +947,21 @@
         <v>20</v>
       </c>
       <c r="C6" s="5"/>
-      <c r="D6" s="38" t="s">
-        <v>21</v>
-      </c>
+      <c r="D6" s="38"/>
       <c r="E6" s="15"/>
-      <c r="F6" s="15">
-        <v>11</v>
-      </c>
+      <c r="F6" s="15"/>
       <c r="G6" s="14"/>
       <c r="H6" s="16"/>
       <c r="I6" s="16"/>
-      <c r="J6" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="K6" s="5">
-        <v>3</v>
-      </c>
-      <c r="L6" s="5">
-        <v>0</v>
-      </c>
+      <c r="J6" s="14"/>
+      <c r="K6" s="5"/>
+      <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5">
-        <v>6.951</v>
+        <v>1.834</v>
       </c>
       <c r="O6" s="5">
-        <v>13.292</v>
+        <v>12.042</v>
       </c>
       <c r="P6" s="10"/>
       <c r="Q6" s="11"/>
@@ -941,7 +980,9 @@
       <c r="A7" s="5">
         <v>3</v>
       </c>
-      <c r="B7" s="13"/>
+      <c r="B7" s="13" t="s">
+        <v>21</v>
+      </c>
       <c r="C7" s="5"/>
       <c r="D7" s="14"/>
       <c r="E7" s="15"/>
@@ -953,8 +994,12 @@
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
-      <c r="N7" s="5"/>
-      <c r="O7" s="5"/>
+      <c r="N7" s="5">
+        <v>2.438</v>
+      </c>
+      <c r="O7" s="5">
+        <v>12.833</v>
+      </c>
       <c r="P7" s="10"/>
       <c r="Q7" s="11"/>
       <c r="R7" s="12"/>
@@ -972,7 +1017,9 @@
       <c r="A8" s="5">
         <v>4</v>
       </c>
-      <c r="B8" s="13"/>
+      <c r="B8" s="13" t="s">
+        <v>22</v>
+      </c>
       <c r="C8" s="5"/>
       <c r="D8" s="14"/>
       <c r="E8" s="15"/>
@@ -984,8 +1031,12 @@
       <c r="K8" s="5"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
-      <c r="N8" s="5"/>
-      <c r="O8" s="5"/>
+      <c r="N8" s="5">
+        <v>10.563</v>
+      </c>
+      <c r="O8" s="5">
+        <v>24.082999999999998</v>
+      </c>
       <c r="P8" s="10"/>
       <c r="Q8" s="11"/>
       <c r="R8" s="12"/>
@@ -1003,7 +1054,9 @@
       <c r="A9" s="5">
         <v>5</v>
       </c>
-      <c r="B9" s="13"/>
+      <c r="B9" s="13" t="s">
+        <v>23</v>
+      </c>
       <c r="C9" s="5"/>
       <c r="D9" s="7"/>
       <c r="E9" s="8"/>
@@ -1015,8 +1068,12 @@
       <c r="K9" s="5"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
-      <c r="N9" s="5"/>
-      <c r="O9" s="5"/>
+      <c r="N9" s="5">
+        <v>58.14</v>
+      </c>
+      <c r="O9" s="5">
+        <v>155.833</v>
+      </c>
       <c r="P9" s="10"/>
       <c r="Q9" s="11"/>
       <c r="R9" s="12"/>
@@ -1034,7 +1091,9 @@
       <c r="A10" s="5">
         <v>6</v>
       </c>
-      <c r="B10" s="13"/>
+      <c r="B10" s="13" t="s">
+        <v>24</v>
+      </c>
       <c r="C10" s="5"/>
       <c r="D10" s="14"/>
       <c r="E10" s="15"/>
@@ -1046,8 +1105,12 @@
       <c r="K10" s="5"/>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
-      <c r="N10" s="5"/>
-      <c r="O10" s="5"/>
+      <c r="N10" s="5">
+        <v>2.618</v>
+      </c>
+      <c r="O10" s="5">
+        <v>12.833</v>
+      </c>
       <c r="P10" s="10"/>
       <c r="Q10" s="11"/>
       <c r="R10" s="12"/>
@@ -1065,7 +1128,9 @@
       <c r="A11" s="5">
         <v>7</v>
       </c>
-      <c r="B11" s="13"/>
+      <c r="B11" s="13" t="s">
+        <v>25</v>
+      </c>
       <c r="C11" s="5"/>
       <c r="D11" s="7"/>
       <c r="E11" s="8"/>
@@ -1077,8 +1142,12 @@
       <c r="K11" s="5"/>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
-      <c r="N11" s="5"/>
-      <c r="O11" s="5"/>
+      <c r="N11" s="5">
+        <v>16.125</v>
+      </c>
+      <c r="O11" s="5">
+        <v>309.5</v>
+      </c>
       <c r="P11" s="10"/>
       <c r="Q11" s="11"/>
       <c r="R11" s="12"/>
@@ -1096,7 +1165,9 @@
       <c r="A12" s="5">
         <v>8</v>
       </c>
-      <c r="B12" s="13"/>
+      <c r="B12" s="13" t="s">
+        <v>26</v>
+      </c>
       <c r="C12" s="5"/>
       <c r="D12" s="14"/>
       <c r="E12" s="15"/>
@@ -1108,8 +1179,12 @@
       <c r="K12" s="5"/>
       <c r="L12" s="5"/>
       <c r="M12" s="5"/>
-      <c r="N12" s="5"/>
-      <c r="O12" s="5"/>
+      <c r="N12" s="5">
+        <v>2.78</v>
+      </c>
+      <c r="O12" s="5">
+        <v>12.958</v>
+      </c>
       <c r="P12" s="10"/>
       <c r="Q12" s="11"/>
       <c r="R12" s="12"/>
@@ -1127,7 +1202,9 @@
       <c r="A13" s="5">
         <v>9</v>
       </c>
-      <c r="B13" s="13"/>
+      <c r="B13" s="13" t="s">
+        <v>27</v>
+      </c>
       <c r="C13" s="5"/>
       <c r="D13" s="14"/>
       <c r="E13" s="15"/>
@@ -1139,8 +1216,12 @@
       <c r="K13" s="5"/>
       <c r="L13" s="5"/>
       <c r="M13" s="5"/>
-      <c r="N13" s="5"/>
-      <c r="O13" s="5"/>
+      <c r="N13" s="5">
+        <v>81.746</v>
+      </c>
+      <c r="O13" s="5">
+        <v>127.75</v>
+      </c>
       <c r="P13" s="10"/>
       <c r="Q13" s="11"/>
       <c r="R13" s="12"/>
@@ -1158,7 +1239,9 @@
       <c r="A14" s="5">
         <v>10</v>
       </c>
-      <c r="B14" s="6"/>
+      <c r="B14" s="6" t="s">
+        <v>28</v>
+      </c>
       <c r="C14" s="5"/>
       <c r="D14" s="14"/>
       <c r="E14" s="15"/>
@@ -1170,8 +1253,12 @@
       <c r="K14" s="5"/>
       <c r="L14" s="5"/>
       <c r="M14" s="5"/>
-      <c r="N14" s="5"/>
-      <c r="O14" s="5"/>
+      <c r="N14" s="5">
+        <v>55.145</v>
+      </c>
+      <c r="O14" s="5">
+        <v>72.082999999999998</v>
+      </c>
       <c r="P14" s="10"/>
       <c r="Q14" s="11"/>
       <c r="R14" s="12"/>
@@ -1189,7 +1276,9 @@
       <c r="A15" s="5">
         <v>11</v>
       </c>
-      <c r="B15" s="13"/>
+      <c r="B15" s="13" t="s">
+        <v>29</v>
+      </c>
       <c r="C15" s="5"/>
       <c r="D15" s="7"/>
       <c r="E15" s="8"/>
@@ -1201,8 +1290,12 @@
       <c r="K15" s="5"/>
       <c r="L15" s="5"/>
       <c r="M15" s="5"/>
-      <c r="N15" s="5"/>
-      <c r="O15" s="5"/>
+      <c r="N15" s="5">
+        <v>91.352</v>
+      </c>
+      <c r="O15" s="5">
+        <v>115.417</v>
+      </c>
       <c r="P15" s="10"/>
       <c r="Q15" s="11"/>
       <c r="R15" s="12"/>
@@ -1220,7 +1313,9 @@
       <c r="A16" s="5">
         <v>12</v>
       </c>
-      <c r="B16" s="13"/>
+      <c r="B16" s="13" t="s">
+        <v>30</v>
+      </c>
       <c r="C16" s="5"/>
       <c r="D16" s="7"/>
       <c r="E16" s="8"/>
@@ -1232,8 +1327,12 @@
       <c r="K16" s="5"/>
       <c r="L16" s="5"/>
       <c r="M16" s="5"/>
-      <c r="N16" s="5"/>
-      <c r="O16" s="5"/>
+      <c r="N16" s="5">
+        <v>73.049999999999997</v>
+      </c>
+      <c r="O16" s="5">
+        <v>114.0</v>
+      </c>
       <c r="P16" s="10"/>
       <c r="Q16" s="11"/>
       <c r="R16" s="12"/>
@@ -1251,7 +1350,9 @@
       <c r="A17" s="5">
         <v>13</v>
       </c>
-      <c r="B17" s="13"/>
+      <c r="B17" s="13" t="s">
+        <v>31</v>
+      </c>
       <c r="C17" s="5"/>
       <c r="D17" s="14"/>
       <c r="E17" s="15"/>
@@ -1263,8 +1364,12 @@
       <c r="K17" s="5"/>
       <c r="L17" s="5"/>
       <c r="M17" s="5"/>
-      <c r="N17" s="5"/>
-      <c r="O17" s="5"/>
+      <c r="N17" s="5">
+        <v>51.825</v>
+      </c>
+      <c r="O17" s="5">
+        <v>70.712</v>
+      </c>
       <c r="P17" s="10"/>
       <c r="Q17" s="11"/>
       <c r="R17" s="12"/>
@@ -1282,7 +1387,9 @@
       <c r="A18" s="5">
         <v>14</v>
       </c>
-      <c r="B18" s="13"/>
+      <c r="B18" s="13" t="s">
+        <v>32</v>
+      </c>
       <c r="C18" s="5"/>
       <c r="D18" s="7"/>
       <c r="E18" s="8"/>
@@ -1294,8 +1401,12 @@
       <c r="K18" s="5"/>
       <c r="L18" s="5"/>
       <c r="M18" s="5"/>
-      <c r="N18" s="5"/>
-      <c r="O18" s="5"/>
+      <c r="N18" s="5">
+        <v>75.729</v>
+      </c>
+      <c r="O18" s="5">
+        <v>101.25</v>
+      </c>
       <c r="P18" s="10"/>
       <c r="Q18" s="11"/>
       <c r="R18" s="12"/>
@@ -1313,7 +1424,9 @@
       <c r="A19" s="5">
         <v>15</v>
       </c>
-      <c r="B19" s="13"/>
+      <c r="B19" s="13" t="s">
+        <v>33</v>
+      </c>
       <c r="C19" s="5"/>
       <c r="D19" s="14"/>
       <c r="E19" s="15"/>
@@ -1325,8 +1438,12 @@
       <c r="K19" s="5"/>
       <c r="L19" s="5"/>
       <c r="M19" s="5"/>
-      <c r="N19" s="5"/>
-      <c r="O19" s="5"/>
+      <c r="N19" s="5">
+        <v>37.894</v>
+      </c>
+      <c r="O19" s="5">
+        <v>54.917</v>
+      </c>
       <c r="P19" s="10"/>
       <c r="Q19" s="11"/>
       <c r="R19" s="12"/>
@@ -1344,7 +1461,9 @@
       <c r="A20" s="5">
         <v>16</v>
       </c>
-      <c r="B20" s="13"/>
+      <c r="B20" s="13" t="s">
+        <v>34</v>
+      </c>
       <c r="C20" s="5"/>
       <c r="D20" s="14"/>
       <c r="E20" s="15"/>
@@ -1356,8 +1475,12 @@
       <c r="K20" s="5"/>
       <c r="L20" s="5"/>
       <c r="M20" s="5"/>
-      <c r="N20" s="5"/>
-      <c r="O20" s="5"/>
+      <c r="N20" s="5">
+        <v>135.37200000000001</v>
+      </c>
+      <c r="O20" s="5">
+        <v>271.54199999999997</v>
+      </c>
       <c r="P20" s="10"/>
       <c r="Q20" s="11"/>
       <c r="R20" s="12"/>
@@ -1375,7 +1498,9 @@
       <c r="A21" s="5">
         <v>17</v>
       </c>
-      <c r="B21" s="13"/>
+      <c r="B21" s="13" t="s">
+        <v>35</v>
+      </c>
       <c r="C21" s="5"/>
       <c r="D21" s="7"/>
       <c r="E21" s="8"/>
@@ -1387,8 +1512,12 @@
       <c r="K21" s="5"/>
       <c r="L21" s="5"/>
       <c r="M21" s="5"/>
-      <c r="N21" s="5"/>
-      <c r="O21" s="5"/>
+      <c r="N21" s="5">
+        <v>78.17100000000001</v>
+      </c>
+      <c r="O21" s="5">
+        <v>123.75</v>
+      </c>
       <c r="P21" s="10"/>
       <c r="Q21" s="11"/>
       <c r="R21" s="12"/>
@@ -1406,7 +1535,9 @@
       <c r="A22" s="5">
         <v>18</v>
       </c>
-      <c r="B22" s="13"/>
+      <c r="B22" s="13" t="s">
+        <v>36</v>
+      </c>
       <c r="C22" s="5"/>
       <c r="D22" s="7"/>
       <c r="E22" s="8"/>
@@ -1418,8 +1549,12 @@
       <c r="K22" s="5"/>
       <c r="L22" s="5"/>
       <c r="M22" s="5"/>
-      <c r="N22" s="5"/>
-      <c r="O22" s="5"/>
+      <c r="N22" s="5">
+        <v>129.102</v>
+      </c>
+      <c r="O22" s="5">
+        <v>260.25</v>
+      </c>
       <c r="P22" s="10"/>
       <c r="Q22" s="11"/>
       <c r="R22" s="12"/>
@@ -1437,7 +1572,9 @@
       <c r="A23" s="5">
         <v>19</v>
       </c>
-      <c r="B23" s="13"/>
+      <c r="B23" s="13" t="s">
+        <v>37</v>
+      </c>
       <c r="C23" s="5"/>
       <c r="D23" s="14"/>
       <c r="E23" s="15"/>
@@ -1449,8 +1586,12 @@
       <c r="K23" s="5"/>
       <c r="L23" s="5"/>
       <c r="M23" s="5"/>
-      <c r="N23" s="5"/>
-      <c r="O23" s="5"/>
+      <c r="N23" s="5">
+        <v>68.419</v>
+      </c>
+      <c r="O23" s="5">
+        <v>128.75</v>
+      </c>
       <c r="P23" s="10"/>
       <c r="Q23" s="11"/>
       <c r="R23" s="12"/>
@@ -1468,7 +1609,9 @@
       <c r="A24" s="5">
         <v>20</v>
       </c>
-      <c r="B24" s="13"/>
+      <c r="B24" s="13" t="s">
+        <v>38</v>
+      </c>
       <c r="C24" s="5"/>
       <c r="D24" s="7"/>
       <c r="E24" s="8"/>
@@ -1480,8 +1623,12 @@
       <c r="K24" s="5"/>
       <c r="L24" s="5"/>
       <c r="M24" s="5"/>
-      <c r="N24" s="5"/>
-      <c r="O24" s="5"/>
+      <c r="N24" s="5">
+        <v>61.363</v>
+      </c>
+      <c r="O24" s="5">
+        <v>128.75</v>
+      </c>
       <c r="P24" s="10"/>
       <c r="Q24" s="11"/>
       <c r="R24" s="12"/>
@@ -1499,7 +1646,9 @@
       <c r="A25" s="5">
         <v>21</v>
       </c>
-      <c r="B25" s="13"/>
+      <c r="B25" s="13" t="s">
+        <v>39</v>
+      </c>
       <c r="C25" s="5"/>
       <c r="D25" s="14"/>
       <c r="E25" s="15"/>
@@ -1511,8 +1660,12 @@
       <c r="K25" s="5"/>
       <c r="L25" s="5"/>
       <c r="M25" s="5"/>
-      <c r="N25" s="5"/>
-      <c r="O25" s="5"/>
+      <c r="N25" s="5">
+        <v>2.766</v>
+      </c>
+      <c r="O25" s="5">
+        <v>12.833</v>
+      </c>
       <c r="P25" s="10"/>
       <c r="Q25" s="11"/>
       <c r="R25" s="12"/>

</xml_diff>